<commit_message>
wrapping sprint 5, starting sprin6 last one
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog6.xlsx
+++ b/presentations/links/sprintbacklog6.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16980"/>
+    <workbookView xWindow="-20" yWindow="460" windowWidth="28800" windowHeight="16980" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Plan and Sprint Report" sheetId="5" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>Task</t>
   </si>
@@ -98,6 +98,39 @@
   </si>
   <si>
     <t>Day 7- Sun Nov 26</t>
+  </si>
+  <si>
+    <t>EXTRAS</t>
+  </si>
+  <si>
+    <t>clean up css</t>
+  </si>
+  <si>
+    <t>bug testing</t>
+  </si>
+  <si>
+    <t>style fix</t>
+  </si>
+  <si>
+    <t>set up one proper assignment with 10 questions</t>
+  </si>
+  <si>
+    <t>refactoring code/ following design patterns</t>
+  </si>
+  <si>
+    <t>Yathan</t>
+  </si>
+  <si>
+    <t>Linhai</t>
+  </si>
+  <si>
+    <t>Jinming</t>
+  </si>
+  <si>
+    <t>Calvn</t>
+  </si>
+  <si>
+    <t>make sure css is responsive as reacts as expected</t>
   </si>
 </sst>
 </file>
@@ -226,15 +259,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -256,6 +283,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="27">
@@ -511,6 +544,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -651,6 +708,30 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -672,11 +753,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-1418168752"/>
-        <c:axId val="-1237622032"/>
+        <c:axId val="-1435809744"/>
+        <c:axId val="-1435806352"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-1418168752"/>
+        <c:axId val="-1435809744"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -775,7 +856,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1237622032"/>
+        <c:crossAx val="-1435806352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -783,7 +864,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-1237622032"/>
+        <c:axId val="-1435806352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -902,7 +983,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1418168752"/>
+        <c:crossAx val="-1435809744"/>
         <c:crossesAt val="1.0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1632,7 +1713,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1949,13 +2030,13 @@
     <col min="7" max="7" width="8.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="2.83203125" style="3" customWidth="1"/>
     <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="15" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="13" customWidth="1"/>
     <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
     <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="6" style="1" customWidth="1"/>
     <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" style="13" customWidth="1"/>
-    <col min="19" max="19" width="7" style="14" customWidth="1"/>
+    <col min="18" max="18" width="3.6640625" style="11" customWidth="1"/>
+    <col min="19" max="19" width="7" style="12" customWidth="1"/>
     <col min="20" max="26" width="6" style="1" customWidth="1"/>
     <col min="27" max="16384" width="12" style="1"/>
   </cols>
@@ -1985,7 +2066,7 @@
       <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="13" t="s">
         <v>11</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -2009,7 +2090,7 @@
       <c r="Q1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="14" t="s">
+      <c r="S1" s="12" t="s">
         <v>12</v>
       </c>
       <c r="T1" s="3" t="s">
@@ -2034,62 +2115,129 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="5"/>
+    <row r="2" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:26" ht="34" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="8"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
+    <row r="3" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="9"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="10"/>
-      <c r="B4" s="5"/>
+    <row r="4" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="9"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="12"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="5"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="5">
+        <v>4</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A6" s="12"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="5"/>
+    <row r="6" spans="1:26" ht="23" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="18"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="5">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="12"/>
-      <c r="B7" s="16"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="5"/>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A8" s="12"/>
-      <c r="B8" s="16"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="5"/>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="12"/>
-      <c r="B9" s="16"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="14"/>
       <c r="C9" s="5"/>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="12"/>
-      <c r="B10" s="16"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="14"/>
     </row>
     <row r="11" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="12"/>
-      <c r="B11" s="16"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="14"/>
       <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="12"/>
-      <c r="B12" s="16"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
@@ -2103,7 +2251,7 @@
       <c r="B16" s="5"/>
       <c r="G16" s="2">
         <f>SUM(G2:G12)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K16" s="6">
         <f>SUM(K1:K12)</f>
@@ -2115,7 +2263,7 @@
       </c>
       <c r="M16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="6">
         <f t="shared" si="0"/>
@@ -2127,7 +2275,7 @@
       </c>
       <c r="P16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="6">
         <f t="shared" si="0"/>
@@ -2181,16 +2329,15 @@
     </row>
     <row r="20" spans="11:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A9:A12"/>
     <mergeCell ref="R1:R1048576"/>
     <mergeCell ref="S1:S1048576"/>
     <mergeCell ref="J1:J1048576"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A5:A6"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B9:B12"/>
+    <mergeCell ref="B2:B6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2209,17 +2356,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2254,22 +2401,70 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2288,10 +2483,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="2:18" ht="26" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="R2" s="8" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2300,10 +2495,7 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -2349,7 +2541,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2358,7 +2550,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
 <xsd:schema targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f7c28edf12e174e47f2c7bd2736e8bd" ns2:_="" ns3:_="" ns4:_="" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d93dc7d-5998-434b-bf34-aa89b432ec07" xmlns:ns3="$ListId:Shared Documents;" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v4">
 <xsd:import namespace="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
 <xsd:import namespace="$ListId:Shared Documents;"/>
@@ -2532,19 +2724,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
-    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
@@ -2552,7 +2735,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2560,7 +2743,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0008E140-BD0E-4C41-947D-F18B1A1E4B6B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2578,4 +2761,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fixed up readme, and main, and some details for sprints
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog6.xlsx
+++ b/presentations/links/sprintbacklog6.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="460" windowWidth="28800" windowHeight="16980" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16980"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Plan and Sprint Report" sheetId="5" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t>Task</t>
   </si>
@@ -115,9 +115,6 @@
     <t>set up one proper assignment with 10 questions</t>
   </si>
   <si>
-    <t>refactoring code/ following design patterns</t>
-  </si>
-  <si>
     <t>Yathan</t>
   </si>
   <si>
@@ -130,7 +127,16 @@
     <t>Calvn</t>
   </si>
   <si>
-    <t>make sure css is responsive as reacts as expected</t>
+    <t>make sure css is responsive as reacts as expected (remove unnecessary stuff) and make the website look nice and usable</t>
+  </si>
+  <si>
+    <t>test all sections of the website, login, student account creation, assignment creation, question creation, student taking a quiz, etc  to make sure it works as expected</t>
+  </si>
+  <si>
+    <t>make sure code is commented and nicely formted</t>
+  </si>
+  <si>
+    <t>clean up existing assignments and questions and make 1 or 2 good assignments for demo purposes</t>
   </si>
 </sst>
 </file>
@@ -242,7 +248,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -263,9 +269,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -275,7 +278,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -283,12 +286,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="27">
@@ -545,22 +542,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0</c:v>
+                  <c:v>10.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.0</c:v>
+                  <c:v>10.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.0</c:v>
+                  <c:v>10.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.0</c:v>
@@ -709,28 +706,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.0</c:v>
+                  <c:v>15.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -753,11 +750,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-1435809744"/>
-        <c:axId val="-1435806352"/>
+        <c:axId val="-808417808"/>
+        <c:axId val="-808372800"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-1435809744"/>
+        <c:axId val="-808417808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -856,7 +853,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1435806352"/>
+        <c:crossAx val="-808372800"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -864,7 +861,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-1435806352"/>
+        <c:axId val="-808372800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -983,7 +980,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1435809744"/>
+        <c:crossAx val="-808417808"/>
         <c:crossesAt val="1.0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1713,7 +1710,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2019,7 +2016,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z20"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
@@ -2030,13 +2027,13 @@
     <col min="7" max="7" width="8.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="2.83203125" style="3" customWidth="1"/>
     <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="13" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="12" customWidth="1"/>
     <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
     <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="6" style="1" customWidth="1"/>
     <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" style="11" customWidth="1"/>
-    <col min="19" max="19" width="7" style="12" customWidth="1"/>
+    <col min="18" max="18" width="3.6640625" style="10" customWidth="1"/>
+    <col min="19" max="19" width="7" style="11" customWidth="1"/>
     <col min="20" max="26" width="6" style="1" customWidth="1"/>
     <col min="27" max="16384" width="12" style="1"/>
   </cols>
@@ -2066,7 +2063,7 @@
       <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>11</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -2090,7 +2087,7 @@
       <c r="Q1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="S1" s="11" t="s">
         <v>12</v>
       </c>
       <c r="T1" s="3" t="s">
@@ -2115,11 +2112,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:26" ht="42" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="17"/>
+      <c r="B2" s="13"/>
       <c r="C2" s="5">
         <v>1</v>
       </c>
@@ -2127,217 +2124,176 @@
         <v>24</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G2" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M2" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:26" ht="47" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="9"/>
-      <c r="B3" s="17"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="5">
         <v>2</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>25</v>
       </c>
+      <c r="E3" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="G3" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P3" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="9"/>
-      <c r="B4" s="17"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="4">
         <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="E4" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="G4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="18"/>
-      <c r="B5" s="17"/>
+    <row r="5" spans="1:26" ht="29" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="9"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="5">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="E5" s="5" t="s">
+        <v>35</v>
+      </c>
       <c r="G5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="23" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="18"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="5">
+    <row r="6" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="7" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" spans="1:26" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="5"/>
+      <c r="G8" s="2">
+        <f>SUM(G2:G5)</f>
+        <v>15</v>
+      </c>
+      <c r="K8" s="6">
+        <f>SUM(K1:K5)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="6">
+        <f>SUM(L2:L5)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="6">
+        <f>SUM(M2:M5)</f>
         <v>5</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="10"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="5"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A8" s="10"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="5"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="10"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="5"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="10"/>
-      <c r="B10" s="14"/>
-    </row>
-    <row r="11" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="10"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="10"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B13" s="5"/>
-    </row>
-    <row r="14" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="15" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="5"/>
-    </row>
-    <row r="16" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="B16" s="5"/>
-      <c r="G16" s="2">
-        <f>SUM(G2:G12)</f>
-        <v>4</v>
-      </c>
-      <c r="K16" s="6">
-        <f>SUM(K1:K12)</f>
+      <c r="N8" s="6">
+        <f>SUM(N2:N5)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="6">
-        <f t="shared" ref="L16:Q16" si="0">SUM(L2:L12)</f>
+      <c r="O8" s="6">
+        <f>SUM(O2:O5)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="6">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="N16" s="6">
+      <c r="P8" s="6">
+        <f>SUM(P2:P5)</f>
+        <v>10</v>
+      </c>
+      <c r="Q8" s="6">
+        <f>SUM(Q2:Q5)</f>
+        <v>0</v>
+      </c>
+      <c r="T8" s="2">
+        <f t="shared" ref="T8:Z8" si="0">SUM(T2:T7)</f>
+        <v>0</v>
+      </c>
+      <c r="U8" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O16" s="6">
+      <c r="V8" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P16" s="6">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="Q16" s="6">
+      <c r="W8" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T16" s="2">
-        <f t="shared" ref="T16:Z16" si="1">SUM(T2:T15)</f>
+      <c r="X8" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="U16" s="2">
-        <f t="shared" si="1"/>
+      <c r="Y8" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="V16" s="2">
-        <f t="shared" si="1"/>
+      <c r="Z8" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="W16" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="X16" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y16" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Z16" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
     </row>
-    <row r="17" spans="11:26" x14ac:dyDescent="0.15">
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="Z17" s="2"/>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="Z9" s="2"/>
     </row>
-    <row r="18" spans="11:26" x14ac:dyDescent="0.15">
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2"/>
     </row>
-    <row r="20" spans="11:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="12" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A9:A12"/>
+  <mergeCells count="5">
     <mergeCell ref="R1:R1048576"/>
     <mergeCell ref="S1:S1048576"/>
     <mergeCell ref="J1:J1048576"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2356,17 +2312,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2402,24 +2358,26 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <f>15-5</f>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H3">
+        <f>10-10</f>
         <v>0</v>
       </c>
       <c r="I3">
@@ -2431,40 +2389,40 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>